<commit_message>
Documents de projet : sécurité renforcée, quittancement, état du 14 octobre
Dossier de conception : règles du quittancement et des pièces déposées,
chapitre sécurité complété (sessions, cloisonnement, approbations,
fichiers, exports, téléphone du parc, politique de contenu). Cahier de
recette : quatre scénarios ajoutés (pièce modifiée après accord,
déconnexion de Rotations, dépôts refusés, cloisonnement d'AxisPro), 59
au total. ETAT.md : troisième revue de sécurité, 97 tests, version
20261014-1502 en production, prochaines étapes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scénarios'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2147,17 +2147,17 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Créer un bien et un bail ; activer le bail.</t>
+          <t>Créer un bien et un bail ; activer le bail ; revenir le lendemain.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Loyer mensuel</t>
+          <t>Loyer mensuel, prise d'effet passée</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Loyers générés depuis la prise d'effet.</t>
+          <t>Chaque nuit, loyers échus depuis la prise d'effet facturés et validés sans intervention (une facture par échéance, datée de l'échéance).</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr"/>
@@ -2631,37 +2631,37 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Grille d'évaluation</t>
+          <t>Achats et dépenses</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
+          <t>Remettre en brouillon une pièce approuvée ; changer le fournisseur ; la valider.</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>Classeur du cabinet</t>
+          <t>Pièce approuvée</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Gates, domaines, 111 critères et pièces chargés ; version 1 en vigueur.</t>
+          <t>Validation refusée : la pièce modifiée repart au circuit d'approbation.</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr"/>
@@ -2673,37 +2673,37 @@
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>R48</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Exploitation</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Dossiers</t>
+          <t>Application Rotations</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Ouvrir un dossier.</t>
+          <t>Se déconnecter ; passer en mode avion ; rouvrir l'application.</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Projet réel anonymisé</t>
+          <t>Saisie en attente</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
+          <t>L'application ne s'ouvre plus sous l'identité de l'agent parti ; sa saisie en attente reste et part à sa prochaine connexion.</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr"/>
@@ -2715,7 +2715,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -2730,22 +2730,22 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Évaluation</t>
+          <t>AxisPro &gt; Grille d'évaluation</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Évaluer les critères ; joindre une preuve pour un critère qui l'exige.</t>
+          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Classeur du cabinet</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Sans preuve, refus ; score et recommandation recalculés.</t>
+          <t>Gates, domaines, 111 critères et pièces chargés ; version 1 en vigueur.</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr"/>
@@ -2757,7 +2757,7 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2772,22 +2772,22 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Synthèse</t>
+          <t>AxisPro &gt; Dossiers</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Contrôler les éliminatoires et les cinq écarts prioritaires ; passer au gate suivant.</t>
+          <t>Ouvrir un dossier.</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Projet réel anonymisé</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>NO-GO si un éliminatoire n'est pas satisfait ; passage refusé tant que le gate n'est pas évalué.</t>
+          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2799,7 +2799,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2814,12 +2814,12 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Comités</t>
+          <t>Dossier &gt; Évaluation</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Enregistrer et verrouiller une décision ; comparer deux revues.</t>
+          <t>Évaluer les critères ; joindre une preuve pour un critère qui l'exige.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Décision non modifiable ; comparaison par domaine.</t>
+          <t>Sans preuve, refus ; score et recommandation recalculés.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr"/>
@@ -2841,7 +2841,7 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Rapport</t>
+          <t>Dossier &gt; Synthèse</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Imprimer le rapport de décision ; l'exporter en XLSX.</t>
+          <t>Contrôler les éliminatoires et les cinq écarts prioritaires ; passer au gate suivant.</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Politique appliquée rappelée ; pièces à fournir listées.</t>
+          <t>NO-GO si un éliminatoire n'est pas satisfait ; passage refusé tant que le gate n'est pas évalué.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2883,7 +2883,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -2898,22 +2898,22 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Temps et facturation</t>
+          <t>Dossier &gt; Comités</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Saisir des temps ; facturer les honoraires.</t>
+          <t>Enregistrer et verrouiller une décision ; comparer deux revues.</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Taux horaire</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
+          <t>Décision non modifiable ; comparaison par domaine.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
@@ -2925,7 +2925,7 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2935,27 +2935,27 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Portail</t>
+          <t>Dossier &gt; Rapport</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+          <t>Imprimer le rapport de décision ; l'exporter en XLSX.</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Accès ouvert par le cabinet</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+          <t>Politique appliquée rappelée ; pièces à fournir listées.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2967,7 +2967,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -2982,22 +2982,22 @@
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Data room</t>
+          <t>Dossier &gt; Temps et facturation</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+          <t>Saisir des temps ; facturer les honoraires.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Taux horaire</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr"/>
@@ -3006,10 +3006,178 @@
       <c r="K56" s="6" t="inlineStr"/>
       <c r="L56" s="6" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Porteur de projet</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Portail</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Accès ouvert par le cabinet</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr"/>
+      <c r="I57" s="7" t="inlineStr"/>
+      <c r="J57" s="7" t="inlineStr"/>
+      <c r="K57" s="7" t="inlineStr"/>
+      <c r="L57" s="7" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>A09</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Data room</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr"/>
+      <c r="I58" s="6" t="inlineStr"/>
+      <c r="J58" s="6" t="inlineStr"/>
+      <c r="K58" s="6" t="inlineStr"/>
+      <c r="L58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Porteur de projet</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Portail &gt; Pièces</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>Fichiers d'essai fournis par le prestataire</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr"/>
+      <c r="I59" s="7" t="inlineStr"/>
+      <c r="J59" s="7" t="inlineStr"/>
+      <c r="K59" s="7" t="inlineStr"/>
+      <c r="L59" s="7" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Direction (société du groupe seule)</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>AxisPro Suite</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr"/>
+      <c r="I60" s="6" t="inlineStr"/>
+      <c r="J60" s="6" t="inlineStr"/>
+      <c r="K60" s="6" t="inlineStr"/>
+      <c r="L60" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L56"/>
+  <autoFilter ref="A1:L60"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
+    <dataValidation sqref="I2:I60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
       <formula1>"OK,KO,Réserve"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3085,19 +3253,19 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"1")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"1")</f>
         <v/>
       </c>
       <c r="D2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"1",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"1",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"1",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"1",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"1",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"1",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G2" s="9">
@@ -3117,19 +3285,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"2")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"2")</f>
         <v/>
       </c>
       <c r="D3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"2",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"2",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"2",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"2",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"2",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"2",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -3149,19 +3317,19 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"3")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"3")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"3",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"3",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"3",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"3",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"3",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"3",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -3181,19 +3349,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"4")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"4")</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"4",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"4",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"4",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"4",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"4",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"4",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3213,19 +3381,19 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"5")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"5")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"5",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"5",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"5",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"5",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"5",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"5",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -3245,19 +3413,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"6")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"6")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"6",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"6",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"6",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"6",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"6",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"6",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3277,19 +3445,19 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"7")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"7")</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"7",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"7",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"7",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"7",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"7",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"7",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -3309,19 +3477,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"8")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"8")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"8",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"8",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"8",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"8",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"8",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"8",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3341,19 +3509,19 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"9")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"9")</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"9",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"9",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"9",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"9",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"9",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"9",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -3373,19 +3541,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"10")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"10")</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"10",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"10",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"10",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"10",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"10",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"10",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3405,19 +3573,19 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"11")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"11")</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"11",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"11",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"11",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"11",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"11",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"11",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -3437,19 +3605,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"12")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"12")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"12",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"12",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"12",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"12",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"12",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"12",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3469,19 +3637,19 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"13")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"13")</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"13",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"13",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"13",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"13",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"13",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"13",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -3501,19 +3669,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"14")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"14")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"14",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"14",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"14",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"14",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"14",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"14",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -3533,19 +3701,19 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"15")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"15")</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"15",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"15",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"15",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"15",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"15",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"15",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -3565,19 +3733,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"16")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"16")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"16",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"16",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"16",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"16",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"16",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"16",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -3597,19 +3765,19 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"17")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"17")</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"17",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"17",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"17",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"17",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"17",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"17",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -3629,19 +3797,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"18")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"18")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"18",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"18",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"18",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"18",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"18",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"18",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -3661,19 +3829,19 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"19")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"19")</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"19",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"19",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"19",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"19",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"19",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"19",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -3693,19 +3861,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$56,"AX")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$60,"AX")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"AX",'Scénarios'!$I$2:$I$56,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"AX",'Scénarios'!$I$2:$I$60,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"AX",'Scénarios'!$I$2:$I$56,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"AX",'Scénarios'!$I$2:$I$60,"Réserve")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$56,"AX",'Scénarios'!$I$2:$I$56,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"AX",'Scénarios'!$I$2:$I$60,"KO")</f>
         <v/>
       </c>
       <c r="G21" s="10">

</xml_diff>

<commit_message>
Cahier de recette et état du projet : fin de bail, intégrité, version 1535
Deux scénarios ajoutés (fin de bail et valorisation d'un bien, contrôles
d'intégrité après clôture), 61 au total. ETAT.md : compléments du
14 octobre et version 20261014-1535 en production.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scénarios'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2715,37 +2715,37 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>R49</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Immobilier</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Grille d'évaluation</t>
+          <t>Immobilier &gt; Biens et baux</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
+          <t>Mettre fin à un bail ; revenir le lendemain ; modifier la valeur actuelle d'un bien.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>Classeur du cabinet</t>
+          <t>Bail en cours</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Gates, domaines, 111 critères et pièces chargés ; version 1 en vigueur.</t>
+          <t>Loyers dus jusqu'à la fin émis, plus aucun ensuite ; bien libre ; valeur et rendement du patrimoine mis à jour.</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr"/>
@@ -2757,37 +2757,37 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>R50</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Dossiers</t>
+          <t>Clôtures et contrôles</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Ouvrir un dossier.</t>
+          <t>Après une clôture mensuelle, consulter les contrôles d'intégrité.</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Projet réel anonymisé</t>
+          <t>Mois clôturé</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
+          <t>Contrôles du mois écoulé et chaînage « Intactes » pour chaque journal verrouillé.</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2799,7 +2799,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2814,22 +2814,22 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Évaluation</t>
+          <t>AxisPro &gt; Grille d'évaluation</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Évaluer les critères ; joindre une preuve pour un critère qui l'exige.</t>
+          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Classeur du cabinet</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Sans preuve, refus ; score et recommandation recalculés.</t>
+          <t>Gates, domaines, 111 critères et pièces chargés ; version 1 en vigueur.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr"/>
@@ -2841,7 +2841,7 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2856,22 +2856,22 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Synthèse</t>
+          <t>AxisPro &gt; Dossiers</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Contrôler les éliminatoires et les cinq écarts prioritaires ; passer au gate suivant.</t>
+          <t>Ouvrir un dossier.</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Projet réel anonymisé</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>NO-GO si un éliminatoire n'est pas satisfait ; passage refusé tant que le gate n'est pas évalué.</t>
+          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2883,7 +2883,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Comités</t>
+          <t>Dossier &gt; Évaluation</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Enregistrer et verrouiller une décision ; comparer deux revues.</t>
+          <t>Évaluer les critères ; joindre une preuve pour un critère qui l'exige.</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Décision non modifiable ; comparaison par domaine.</t>
+          <t>Sans preuve, refus ; score et recommandation recalculés.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
@@ -2925,7 +2925,7 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2940,12 +2940,12 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Rapport</t>
+          <t>Dossier &gt; Synthèse</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Imprimer le rapport de décision ; l'exporter en XLSX.</t>
+          <t>Contrôler les éliminatoires et les cinq écarts prioritaires ; passer au gate suivant.</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Politique appliquée rappelée ; pièces à fournir listées.</t>
+          <t>NO-GO si un éliminatoire n'est pas satisfait ; passage refusé tant que le gate n'est pas évalué.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2967,7 +2967,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -2982,22 +2982,22 @@
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Temps et facturation</t>
+          <t>Dossier &gt; Comités</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Saisir des temps ; facturer les honoraires.</t>
+          <t>Enregistrer et verrouiller une décision ; comparer deux revues.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>Taux horaire</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
+          <t>Décision non modifiable ; comparaison par domaine.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr"/>
@@ -3009,7 +3009,7 @@
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3019,27 +3019,27 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Portail</t>
+          <t>Dossier &gt; Rapport</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+          <t>Imprimer le rapport de décision ; l'exporter en XLSX.</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Accès ouvert par le cabinet</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+          <t>Politique appliquée rappelée ; pièces à fournir listées.</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3051,7 +3051,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -3066,22 +3066,22 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Data room</t>
+          <t>Dossier &gt; Temps et facturation</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+          <t>Saisir des temps ; facturer les honoraires.</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Taux horaire</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr"/>
@@ -3093,7 +3093,7 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3108,22 +3108,22 @@
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Portail &gt; Pièces</t>
+          <t>Portail</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Fichiers d'essai fournis par le prestataire</t>
+          <t>Accès ouvert par le cabinet</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3135,7 +3135,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>A09</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -3145,17 +3145,17 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Direction (société du groupe seule)</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>AxisPro Suite</t>
+          <t>Dossier &gt; Data room</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -3174,10 +3174,94 @@
       <c r="K60" s="6" t="inlineStr"/>
       <c r="L60" s="6" t="inlineStr"/>
     </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Porteur de projet</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Portail &gt; Pièces</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Fichiers d'essai fournis par le prestataire</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr"/>
+      <c r="I61" s="7" t="inlineStr"/>
+      <c r="J61" s="7" t="inlineStr"/>
+      <c r="K61" s="7" t="inlineStr"/>
+      <c r="L61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Direction (société du groupe seule)</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>AxisPro Suite</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr"/>
+      <c r="I62" s="6" t="inlineStr"/>
+      <c r="J62" s="6" t="inlineStr"/>
+      <c r="K62" s="6" t="inlineStr"/>
+      <c r="L62" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L60"/>
+  <autoFilter ref="A1:L62"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
+    <dataValidation sqref="I2:I62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
       <formula1>"OK,KO,Réserve"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3253,19 +3337,19 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"1")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"1")</f>
         <v/>
       </c>
       <c r="D2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"1",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"1",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"1",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"1",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"1",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"1",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G2" s="9">
@@ -3285,19 +3369,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"2")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"2")</f>
         <v/>
       </c>
       <c r="D3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"2",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"2",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"2",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"2",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"2",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"2",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -3317,19 +3401,19 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"3")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"3")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"3",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"3",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"3",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"3",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"3",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"3",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -3349,19 +3433,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"4")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"4")</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"4",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"4",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"4",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"4",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"4",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"4",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3381,19 +3465,19 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"5")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"5")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"5",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"5",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"5",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"5",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"5",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"5",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -3413,19 +3497,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"6")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"6")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"6",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"6",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"6",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"6",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"6",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"6",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3445,19 +3529,19 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"7")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"7")</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"7",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"7",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"7",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"7",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"7",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"7",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -3477,19 +3561,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"8")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"8")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"8",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"8",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"8",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"8",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"8",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"8",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3509,19 +3593,19 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"9")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"9")</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"9",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"9",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"9",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"9",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"9",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"9",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -3541,19 +3625,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"10")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"10")</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"10",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"10",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"10",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"10",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"10",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"10",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3573,19 +3657,19 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"11")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"11")</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"11",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"11",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"11",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"11",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"11",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"11",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -3605,19 +3689,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"12")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"12")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"12",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"12",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"12",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"12",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"12",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"12",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3637,19 +3721,19 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"13")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"13")</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"13",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"13",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"13",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"13",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"13",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"13",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -3669,19 +3753,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"14")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"14")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"14",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"14",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"14",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"14",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"14",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"14",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -3701,19 +3785,19 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"15")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"15")</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"15",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"15",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"15",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"15",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"15",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"15",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -3733,19 +3817,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"16")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"16")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"16",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"16",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"16",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"16",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"16",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"16",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -3765,19 +3849,19 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"17")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"17")</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"17",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"17",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"17",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"17",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"17",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"17",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -3797,19 +3881,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"18")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"18")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"18",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"18",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"18",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"18",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"18",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"18",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -3829,19 +3913,19 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"19")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"19")</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"19",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"19",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"19",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"19",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"19",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"19",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -3861,19 +3945,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$60,"AX")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$62,"AX")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"AX",'Scénarios'!$I$2:$I$60,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"AX",'Scénarios'!$I$2:$I$62,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"AX",'Scénarios'!$I$2:$I$60,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"AX",'Scénarios'!$I$2:$I$62,"Réserve")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$60,"AX",'Scénarios'!$I$2:$I$60,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"AX",'Scénarios'!$I$2:$I$62,"KO")</f>
         <v/>
       </c>
       <c r="G21" s="10">

</xml_diff>

<commit_message>
Cahier de recette : méthode MB AxisPro, restauration avec compte rendu, support, dossier technique
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Restaurer la production à un instant choisi dans un environnement jetable.</t>
+          <t>Restaurer la production à un instant choisi dans un environnement jetable (backup/restore-test.sh --target … --report).</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Base restaurée et contrôlée (sociétés, pièces) ; compte rendu remis.</t>
+          <t>Base restaurée et contrôlée (sociétés, pièces) ; compte rendu remis ; disponibilité du mois écoulé calculée (availability-report.py).</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr"/>
@@ -2567,17 +2567,17 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Déclarer une anomalie de recette.</t>
+          <t>Déclarer une anomalie de recette selon la procédure de support.</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Procédure de support remise</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Prise en compte dans les délais de l'offre (chapitre 7.2).</t>
+          <t>Accusé de réception, gravité confirmée, prise en compte dans les délais de l'offre (chapitre 7.2).</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr"/>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Installer une évolution en recette, la faire valider, la mettre en production.</t>
+          <t>Ajouter une fonction ou un module du noyau selon le dossier technique, l'installer en recette, la faire valider, la mettre en production.</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dossier technique</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Gates, domaines, 111 critères et pièces chargés ; version 1 en vigueur.</t>
+          <t>8 gates et leurs règles, 15 domaines, 111 critères (9 knock-outs), 42 pièces et 102 rattachements chargés ; version en vigueur.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr"/>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Évaluer les critères ; joindre une preuve pour un critère qui l'exige.</t>
+          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Sans preuve, refus ; score et recommandation recalculés.</t>
+          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Contrôler les éliminatoires et les cinq écarts prioritaires ; passer au gate suivant.</t>
+          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>NO-GO si un éliminatoire n'est pas satisfait ; passage refusé tant que le gate n'est pas évalué.</t>
+          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Enregistrer et verrouiller une décision ; comparer deux revues.</t>
+          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Décision non modifiable ; comparaison par domaine.</t>
+          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr"/>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Imprimer le rapport de décision ; l'exporter en XLSX.</t>
+          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Politique appliquée rappelée ; pièces à fournir listées.</t>
+          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Cahier de recette : douze scénarios des prototypes de la direction (consolidé, questions du dirigeant, engagements, décaissements, clôture complète, validation n/26, camt.053)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$74</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scénarios'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Importer un relevé bancaire réel (CSV ou XLSX).</t>
+          <t>Importer un relevé bancaire réel (CSV, XLSX ou camt.053 XML) ; réimporter le même fichier.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Lignes importées, doublons refusés, solde conforme au relevé.</t>
+          <t>Lignes importées, soldes initial et final lus et contrôlés (écart refusé sauf confirmation), doublons ignorés à la réimportation.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr"/>
@@ -2799,37 +2799,37 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Direction</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Grille d'évaluation</t>
+          <t>Balance et états &gt; Consolidé du groupe</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
+          <t>Facturer une prestation d'une société du groupe à l'autre ; afficher le consolidé de l'exercice.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Classeur du cabinet</t>
+          <t>Facture intra-groupe</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>8 gates et leurs règles, 15 domaines, 111 critères (9 knock-outs), 42 pièces et 102 rattachements chargés ; version en vigueur.</t>
+          <t>Compte de résultat et bilan par société ; la vente et l'achat réciproques, la créance et la dette s'éliminent ; colonne Groupe = somme des sociétés − éliminations.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr"/>
@@ -2841,37 +2841,37 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>R52</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Direction</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Dossiers</t>
+          <t>Finance &gt; Tableau de bord</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Ouvrir un dossier.</t>
+          <t>Choisir une date d'arrêté ; lire les onze questions du dirigeant et le bloc « Ce qui demande une décision » ; imprimer.</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Projet réel anonymisé</t>
+          <t>Données reprises</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
+          <t>Chaque question a sa réponse, son verdict (vert, orange, rouge) et sa lecture ; décisions reliées aux alertes.</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2883,27 +2883,27 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>R53</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Évaluation</t>
+          <t>Pilotage &gt; Alertes</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
+          <t>Afficher toutes les règles, conformes comprises ; modifier un seuil (DSCR, délai de recouvrement).</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
+          <t>Gravité, valeur, seuil et action recommandée pour chaque règle ; seuil laissé à zéro signalé en vigilance.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
@@ -2925,37 +2925,37 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>R54</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Synthèse</t>
+          <t>Achats et dépenses</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
+          <t>Saisir une dépense par sa catégorie, sur deux axes (activité et ensemble routier).</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Catégorie Carburant</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
+          <t>Compte de charge, compte du fournisseur et TVA déduits de la catégorie ; ventilation analytique sur les deux axes.</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2967,37 +2967,37 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>R55</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Comités</t>
+          <t>Activités et budget &gt; Budget</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
+          <t>Importer le budget par ligne budgétaire (XLSX) ; comparer au réalisé et aux engagements.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Budget 2026 du classeur</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
+          <t>Budget cumulé, réalisé, engagé, disponible, écart et statut (dépassement, conforme, sous-réalisation) par ligne.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr"/>
@@ -3009,37 +3009,37 @@
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Chantiers puis finance et direction</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Rapport</t>
+          <t>Engagements</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
+          <t>Créer un engagement de dépense de 60 M GNF avec son devis ; le faire approuver ; saisir ensuite la facture du fournisseur.</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Devis joint</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
+          <t>Engagement approuvé par la finance puis la direction ; la facture consomme l'engagement sans refaire le circuit ; reste à engager à jour.</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3051,37 +3051,37 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>R57</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance puis direction</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Temps et facturation</t>
+          <t>Trésorerie</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Saisir des temps ; facturer les honoraires.</t>
+          <t>Saisir une sortie de banque de 150 M GNF ; tenter de la comptabiliser.</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>Taux horaire</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
+          <t>Opération en brouillon jusqu'à l'accord de la direction, comptabilisée à la dernière approbation.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr"/>
@@ -3093,37 +3093,37 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>R58</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Portail</t>
+          <t>Clôtures et contrôles &gt; Clôture mensuelle</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+          <t>Clôturer un mois complet.</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Accès ouvert par le cabinet</t>
+          <t>Mois repris</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+          <t>Dotations, liquidation de la TVA (pièce TVA du mois), factures à établir des rotations non facturées (extournées le mois suivant), sceau et procès-verbal imprimé.</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3135,37 +3135,37 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance et responsable financier</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Data room</t>
+          <t>Clôtures et contrôles &gt; Validation de la reprise</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+          <t>Charger les valeurs de référence du classeur ; lancer le contrôle ; imprimer l'annexe.</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Valeurs de référence du classeur</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+          <t>26 indicateurs recalculés, écart de chacun ; « 26/26 » conformes attendu avant la bascule ; annexe jointe au procès-verbal de bascule.</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -3177,37 +3177,37 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>R60</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Direction</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Portail &gt; Pièces</t>
+          <t>Transport &gt; Rentabilité</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+          <t>Afficher la rentabilité par ensemble routier avec les charges de structure ; contrôler les manquants d'une rotation.</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Fichiers d'essai fournis par le prestataire</t>
+          <t>Rotations reprises</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+          <t>Coût et CA au km, structure, résultat net par ensemble ; manquant toléré, excédentaire déduit ou imputé au chauffeur ; taxes spécifiques au barème.</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3219,37 +3219,37 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>R61</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Direction (société du groupe seule)</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>AxisPro Suite</t>
+          <t>Fiscalité</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+          <t>Saisir une facture fournisseur soumise à retenue à la source ; consulter la déclaration du mois.</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Prestataire non résident ou retenue BIC</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+          <t>Retenue calculée et portée au compte de l'État ; déclaration et historique à jour.</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3258,10 +3258,514 @@
       <c r="K62" s="6" t="inlineStr"/>
       <c r="L62" s="6" t="inlineStr"/>
     </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>R62</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Pilotage &gt; Trésorerie</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Afficher les flux mensuels et la prévision ; régler une échéance d'emprunt depuis une ligne de relevé.</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Emprunt repris</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>Encaissements, décaissements, cash net et solde par mois face au seuil ; échéance proposée au rapprochement, capital et intérêts comptabilisés une seule fois.</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr"/>
+      <c r="I63" s="7" t="inlineStr"/>
+      <c r="J63" s="7" t="inlineStr"/>
+      <c r="K63" s="7" t="inlineStr"/>
+      <c r="L63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>AxisPro &gt; Grille d'évaluation</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Classeur du cabinet</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>8 gates et leurs règles, 15 domaines, 111 critères (9 knock-outs), 42 pièces et 102 rattachements chargés ; version en vigueur.</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr"/>
+      <c r="I64" s="6" t="inlineStr"/>
+      <c r="J64" s="6" t="inlineStr"/>
+      <c r="K64" s="6" t="inlineStr"/>
+      <c r="L64" s="6" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>AxisPro &gt; Dossiers</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Ouvrir un dossier.</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>Projet réel anonymisé</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr"/>
+      <c r="I65" s="7" t="inlineStr"/>
+      <c r="J65" s="7" t="inlineStr"/>
+      <c r="K65" s="7" t="inlineStr"/>
+      <c r="L65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Évaluation</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr"/>
+      <c r="I66" s="6" t="inlineStr"/>
+      <c r="J66" s="6" t="inlineStr"/>
+      <c r="K66" s="6" t="inlineStr"/>
+      <c r="L66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Synthèse</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr"/>
+      <c r="I67" s="7" t="inlineStr"/>
+      <c r="J67" s="7" t="inlineStr"/>
+      <c r="K67" s="7" t="inlineStr"/>
+      <c r="L67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Comités</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr"/>
+      <c r="I68" s="6" t="inlineStr"/>
+      <c r="J68" s="6" t="inlineStr"/>
+      <c r="K68" s="6" t="inlineStr"/>
+      <c r="L68" s="6" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Rapport</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr"/>
+      <c r="I69" s="7" t="inlineStr"/>
+      <c r="J69" s="7" t="inlineStr"/>
+      <c r="K69" s="7" t="inlineStr"/>
+      <c r="L69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Temps et facturation</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>Saisir des temps ; facturer les honoraires.</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>Taux horaire</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr"/>
+      <c r="I70" s="6" t="inlineStr"/>
+      <c r="J70" s="6" t="inlineStr"/>
+      <c r="K70" s="6" t="inlineStr"/>
+      <c r="L70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Porteur de projet</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Portail</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>Accès ouvert par le cabinet</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr"/>
+      <c r="I71" s="7" t="inlineStr"/>
+      <c r="J71" s="7" t="inlineStr"/>
+      <c r="K71" s="7" t="inlineStr"/>
+      <c r="L71" s="7" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>A09</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Data room</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr"/>
+      <c r="I72" s="6" t="inlineStr"/>
+      <c r="J72" s="6" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr"/>
+      <c r="L72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Porteur de projet</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Portail &gt; Pièces</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>Fichiers d'essai fournis par le prestataire</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr"/>
+      <c r="I73" s="7" t="inlineStr"/>
+      <c r="J73" s="7" t="inlineStr"/>
+      <c r="K73" s="7" t="inlineStr"/>
+      <c r="L73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Direction (société du groupe seule)</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>AxisPro Suite</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr"/>
+      <c r="I74" s="6" t="inlineStr"/>
+      <c r="J74" s="6" t="inlineStr"/>
+      <c r="K74" s="6" t="inlineStr"/>
+      <c r="L74" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L62"/>
+  <autoFilter ref="A1:L74"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
+    <dataValidation sqref="I2:I74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
       <formula1>"OK,KO,Réserve"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3337,19 +3841,19 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"1")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"1")</f>
         <v/>
       </c>
       <c r="D2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"1",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"1",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"1",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"1",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"1",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"1",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G2" s="9">
@@ -3369,19 +3873,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"2")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"2")</f>
         <v/>
       </c>
       <c r="D3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"2",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"2",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"2",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"2",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"2",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"2",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -3401,19 +3905,19 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"3")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"3")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"3",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"3",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"3",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"3",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"3",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"3",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -3433,19 +3937,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"4")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"4")</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"4",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"4",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"4",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"4",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"4",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"4",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3465,19 +3969,19 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"5")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"5")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"5",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"5",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"5",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"5",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"5",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"5",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -3497,19 +4001,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"6")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"6")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"6",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"6",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"6",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"6",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"6",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"6",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3529,19 +4033,19 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"7")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"7")</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"7",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"7",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"7",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"7",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"7",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"7",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -3561,19 +4065,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"8")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"8")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"8",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"8",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"8",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"8",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"8",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"8",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3593,19 +4097,19 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"9")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"9")</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"9",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"9",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"9",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"9",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"9",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"9",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -3625,19 +4129,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"10")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"10")</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"10",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"10",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"10",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"10",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"10",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"10",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3657,19 +4161,19 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"11")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"11")</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"11",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"11",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"11",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"11",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"11",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"11",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -3689,19 +4193,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"12")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"12")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"12",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"12",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"12",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"12",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"12",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"12",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3721,19 +4225,19 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"13")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"13")</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"13",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"13",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"13",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"13",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"13",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"13",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -3753,19 +4257,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"14")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"14")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"14",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"14",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"14",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"14",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"14",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"14",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -3785,19 +4289,19 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"15")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"15")</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"15",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"15",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"15",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"15",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"15",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"15",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -3817,19 +4321,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"16")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"16")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"16",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"16",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"16",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"16",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"16",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"16",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -3849,19 +4353,19 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"17")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"17")</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"17",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"17",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"17",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"17",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"17",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"17",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -3881,19 +4385,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"18")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"18")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"18",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"18",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"18",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"18",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"18",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"18",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -3913,19 +4417,19 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"19")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"19")</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"19",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"19",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"19",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"19",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"19",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"19",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -3945,19 +4449,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$62,"AX")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$74,"AX")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"AX",'Scénarios'!$I$2:$I$62,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"AX",'Scénarios'!$I$2:$I$74,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"AX",'Scénarios'!$I$2:$I$62,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"AX",'Scénarios'!$I$2:$I$74,"Réserve")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$62,"AX",'Scénarios'!$I$2:$I$62,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"AX",'Scénarios'!$I$2:$I$74,"KO")</f>
         <v/>
       </c>
       <c r="G21" s="10">

</xml_diff>

<commit_message>
La société du cabinet devient « MB AxisPro » ; le métier « Chantiers » devient « BTP »
Décisions du gérant du 21 octobre. Nom de la société dans le code, les écrans, la maquette, les guides
et les documents de projet (l'offre et l'accord de confidentialité signés restent inchangés) ; migration
d'eguitra_base 19.0.1.3.0 qui renomme la société du cabinet dans les bases existantes. Libellés du
profil, du module, du menu et des analyses : « BTP » (un chantier reste un chantier).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Passer d'EGUITRA GROUP SARLU à MB AxisPro Consulting, puis revenir.</t>
+          <t>Passer d'EGUITRA GROUP SARLU à MB AxisPro, puis revenir.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Le premier voit le sélecteur et les deux sociétés ; le second ne voit que MB AxisPro Consulting.</t>
+          <t>Le premier voit le sélecteur et les deux sociétés ; le second ne voit que MB AxisPro.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
Transport : ensembles gérés pour des propriétaires, relevés et coûts standard
Noyau (eguitra_transport 19.0.1.3.0) : propriété des ensembles (propre ou
géré pour un propriétaire) et charges mensuelles ; règles de répartition en
pourcentage du chiffre d'affaires brut, par ensemble ou par catégorie ;
relevés par ensemble et par période (frais déclarés et charges mensuelles,
ou pièces comptabilisées), PDF et Excel, pièces en brouillon (part du
propriétaire, refacturation d'une part négative, commissions des tiers).
Coûts standard des routes et prix du carburant datés : coût standard et
marge estimée des rotations, figés à la validation ; rentabilité et
contrôle des forfaits incohérents. Piste d'audit étendue ; 10 tests.

Web : onglet Propriétaires, propriété et charges dans la flotte, forfaits
et prix du carburant dans les routes, gain estimé à la saisie, paramètres
des relevés. Maquette d'API complétée pour ces écrans.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$77</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scénarios'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3261,12 +3261,12 @@
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>R62</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -3276,22 +3276,22 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Pilotage &gt; Trésorerie</t>
+          <t>Transport &gt; Routes et tarifs</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Afficher les flux mensuels et la prévision ; régler une échéance d'emprunt depuis une ligne de relevé.</t>
+          <t>Renseigner les forfaits d'une route et le prix du carburant ; saisir une rotation, la valider, puis changer le prix.</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Emprunt repris</t>
+          <t>Route et ensemble existants</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Encaissements, décaissements, cash net et solde par mois face au seuil ; échéance proposée au rapprochement, capital et intérêts comptabilisés une seule fois.</t>
+          <t>Coût standard et marge estimée affichés à la saisie ; après validation, un nouveau prix ne change pas la rotation ; rentabilité : coûts standard, déclarés et comptabilisés côte à côte.</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3303,37 +3303,37 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>R64</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Grille d'évaluation</t>
+          <t>Transport &gt; Flotte, Propriétaires</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
+          <t>Déclarer un ensemble géré pour un propriétaire avec ses charges mensuelles ; créer une règle de 5 % pour la société et une commission de partenaire ; établir les relevés du mois.</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>Classeur du cabinet</t>
+          <t>Rotations validées sur l'ensemble</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>8 gates et leurs règles, 15 domaines, 111 critères (9 knock-outs), 42 pièces et 102 rattachements chargés ; version en vigueur.</t>
+          <t>Relevé : chiffre d'affaires, charges, marge, commissions, part du propriétaire ; PDF et Excel ; ensemble à l'arrêt : part négative.</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -3345,37 +3345,37 @@
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>R65</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Dossiers</t>
+          <t>Transport &gt; Propriétaires</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Ouvrir un dossier.</t>
+          <t>Préparer les pièces d'un relevé, les consulter dans Achats et Ventes, puis rouvrir le relevé.</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Projet réel anonymisé</t>
+          <t>Relevé établi</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
+          <t>Facture d'achat du propriétaire (ou refacturation d'une part négative) et facture du partenaire en brouillon, imputées sur l'ensemble ; aucune pièce pour la part de la société ; rouvrir supprime les brouillons.</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3387,37 +3387,37 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>R62</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Évaluation</t>
+          <t>Pilotage &gt; Trésorerie</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
+          <t>Afficher les flux mensuels et la prévision ; régler une échéance d'emprunt depuis une ligne de relevé.</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Emprunt repris</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
+          <t>Encaissements, décaissements, cash net et solde par mois face au seuil ; échéance proposée au rapprochement, capital et intérêts comptabilisés une seule fois.</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3429,7 +3429,7 @@
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3444,22 +3444,22 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Synthèse</t>
+          <t>AxisPro &gt; Grille d'évaluation</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
+          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Classeur du cabinet</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
+          <t>8 gates et leurs règles, 15 domaines, 111 critères (9 knock-outs), 42 pièces et 102 rattachements chargés ; version en vigueur.</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3471,7 +3471,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -3486,22 +3486,22 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Comités</t>
+          <t>AxisPro &gt; Dossiers</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
+          <t>Ouvrir un dossier.</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Projet réel anonymisé</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
+          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3513,7 +3513,7 @@
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3528,12 +3528,12 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Rapport</t>
+          <t>Dossier &gt; Évaluation</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
+          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
+          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3555,7 +3555,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -3570,22 +3570,22 @@
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Temps et facturation</t>
+          <t>Dossier &gt; Synthèse</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Saisir des temps ; facturer les honoraires.</t>
+          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>Taux horaire</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
+          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
@@ -3597,7 +3597,7 @@
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3607,27 +3607,27 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Portail</t>
+          <t>Dossier &gt; Comités</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Accès ouvert par le cabinet</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3639,7 +3639,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -3654,12 +3654,12 @@
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Data room</t>
+          <t>Dossier &gt; Rapport</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
@@ -3681,7 +3681,7 @@
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3691,27 +3691,27 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Portail &gt; Pièces</t>
+          <t>Dossier &gt; Temps et facturation</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+          <t>Saisir des temps ; facturer les honoraires.</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>Fichiers d'essai fournis par le prestataire</t>
+          <t>Taux horaire</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3723,7 +3723,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -3733,27 +3733,27 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Direction (société du groupe seule)</t>
+          <t>Porteur de projet</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>AxisPro Suite</t>
+          <t>Portail</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Accès ouvert par le cabinet</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -3762,10 +3762,136 @@
       <c r="K74" s="6" t="inlineStr"/>
       <c r="L74" s="6" t="inlineStr"/>
     </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>A09</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Data room</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr"/>
+      <c r="I75" s="7" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr"/>
+      <c r="K75" s="7" t="inlineStr"/>
+      <c r="L75" s="7" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Porteur de projet</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Portail &gt; Pièces</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>Fichiers d'essai fournis par le prestataire</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr"/>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="inlineStr"/>
+      <c r="K76" s="6" t="inlineStr"/>
+      <c r="L76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Direction (société du groupe seule)</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>AxisPro Suite</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr"/>
+      <c r="I77" s="7" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr"/>
+      <c r="K77" s="7" t="inlineStr"/>
+      <c r="L77" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L74"/>
+  <autoFilter ref="A1:L77"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
+    <dataValidation sqref="I2:I77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
       <formula1>"OK,KO,Réserve"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3841,19 +3967,19 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"1")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"1")</f>
         <v/>
       </c>
       <c r="D2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"1",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"1",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"1",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"1",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"1",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"1",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G2" s="9">
@@ -3873,19 +3999,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"2")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"2")</f>
         <v/>
       </c>
       <c r="D3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"2",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"2",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"2",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"2",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"2",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"2",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -3905,19 +4031,19 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"3")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"3")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"3",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"3",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"3",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"3",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"3",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"3",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -3937,19 +4063,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"4")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"4")</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"4",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"4",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"4",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"4",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"4",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"4",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3969,19 +4095,19 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"5")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"5")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"5",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"5",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"5",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"5",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"5",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"5",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -4001,19 +4127,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"6")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"6")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"6",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"6",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"6",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"6",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"6",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"6",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4033,19 +4159,19 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"7")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"7")</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"7",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"7",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"7",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"7",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"7",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"7",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -4065,19 +4191,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"8")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"8")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"8",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"8",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"8",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"8",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"8",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"8",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4097,19 +4223,19 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"9")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"9")</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"9",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"9",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"9",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"9",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"9",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"9",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -4129,19 +4255,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"10")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"10")</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"10",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"10",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"10",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"10",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"10",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"10",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4161,19 +4287,19 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"11")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"11")</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"11",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"11",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"11",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"11",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"11",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"11",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -4193,19 +4319,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"12")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"12")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"12",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"12",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"12",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"12",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"12",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"12",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4225,19 +4351,19 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"13")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"13")</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"13",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"13",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"13",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"13",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"13",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"13",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -4257,19 +4383,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"14")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"14")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"14",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"14",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"14",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"14",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"14",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"14",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4289,19 +4415,19 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"15")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"15")</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"15",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"15",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"15",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"15",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"15",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"15",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -4321,19 +4447,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"16")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"16")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"16",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"16",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"16",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"16",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"16",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"16",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -4353,19 +4479,19 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"17")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"17")</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"17",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"17",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"17",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"17",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"17",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"17",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -4385,19 +4511,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"18")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"18")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"18",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"18",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"18",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"18",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"18",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"18",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -4417,19 +4543,19 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"19")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"19")</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"19",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"19",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"19",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"19",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"19",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"19",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -4449,19 +4575,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$74,"AX")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$77,"AX")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"AX",'Scénarios'!$I$2:$I$74,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"AX",'Scénarios'!$I$2:$I$77,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"AX",'Scénarios'!$I$2:$I$74,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"AX",'Scénarios'!$I$2:$I$77,"Réserve")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$74,"AX",'Scénarios'!$I$2:$I$74,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"AX",'Scénarios'!$I$2:$I$77,"KO")</f>
         <v/>
       </c>
       <c r="G21" s="10">

</xml_diff>

<commit_message>
Guide du cabinet et cahier de recette : outil de scoring v3, compartiments, complétude d'entrée des gates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$80</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scénarios'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3449,17 +3449,17 @@
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Importer la grille officielle ; la vérifier ; la mettre en vigueur.</t>
+          <t>Importer l'outil de scoring du cabinet tel quel (version 3) ; le vérifier ; le mettre en vigueur.</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Classeur du cabinet</t>
+          <t>Outil de scoring du cabinet (classeur)</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>8 gates et leurs règles, 15 domaines, 111 critères (9 knock-outs), 42 pièces et 102 rattachements chargés ; version en vigueur.</t>
+          <t>7 gates et leurs règles (complétude minimale de 40 % au gate 1), 8 compartiments, 14 domaines, 104 critères (9 knock-outs), 39 pièces rattachées ; codes repris de la version précédente ; knock-out incomplet non bloquant, non applicable à 1 point ; version en vigueur.</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3888,10 +3888,136 @@
       <c r="K77" s="7" t="inlineStr"/>
       <c r="L77" s="7" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Synthèse, Évaluation</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>Confier deux compartiments à deux consultants ; filtrer la check-list sur « Mes compartiments » avec chacun.</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>Deux comptes cabinet</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>Suivi par compartiment : score, critères, manques, études renseignées, consultant ; chaque consultant ne voit que ses critères ; changements inscrits au journal.</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
+      <c r="I78" s="6" t="inlineStr"/>
+      <c r="J78" s="6" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr"/>
+      <c r="L78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>A13</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Stage gates</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Évaluer quelques critères du gate 1 en dessous de 40 % de complétude, puis au-dessus.</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>Dossier ouvert</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>Gate 1 en HOLD avec le motif de complétude, puis GO ou CONDITIONAL GO selon le score.</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr"/>
+      <c r="I79" s="7" t="inlineStr"/>
+      <c r="J79" s="7" t="inlineStr"/>
+      <c r="K79" s="7" t="inlineStr"/>
+      <c r="L79" s="7" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Évaluation &gt; Importer une fiche</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>Remplir l'outil de scoring du cabinet hors ligne (statuts, études à produire) et l'importer dans un dossier.</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>Outil du cabinet rempli</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>Aperçu des changements, puis statuts et études à produire repris ; notices de l'outil ignorées.</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr"/>
+      <c r="I80" s="6" t="inlineStr"/>
+      <c r="J80" s="6" t="inlineStr"/>
+      <c r="K80" s="6" t="inlineStr"/>
+      <c r="L80" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L77"/>
+  <autoFilter ref="A1:L80"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
+    <dataValidation sqref="I2:I80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
       <formula1>"OK,KO,Réserve"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3967,19 +4093,19 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"1")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"1")</f>
         <v/>
       </c>
       <c r="D2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"1",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"1",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"1",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"1",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"1",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"1",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G2" s="9">
@@ -3999,19 +4125,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"2")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"2")</f>
         <v/>
       </c>
       <c r="D3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"2",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"2",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"2",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"2",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"2",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"2",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -4031,19 +4157,19 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"3")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"3")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"3",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"3",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"3",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"3",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"3",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"3",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -4063,19 +4189,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"4")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"4")</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"4",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"4",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"4",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"4",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"4",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"4",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4095,19 +4221,19 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"5")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"5")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"5",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"5",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"5",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"5",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"5",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"5",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -4127,19 +4253,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"6")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"6")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"6",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"6",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"6",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"6",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"6",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"6",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4159,19 +4285,19 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"7")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"7")</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"7",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"7",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"7",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"7",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"7",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"7",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -4191,19 +4317,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"8")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"8")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"8",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"8",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"8",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"8",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"8",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"8",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4223,19 +4349,19 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"9")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"9")</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"9",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"9",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"9",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"9",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"9",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"9",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -4255,19 +4381,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"10")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"10")</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"10",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"10",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"10",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"10",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"10",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"10",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4287,19 +4413,19 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"11")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"11")</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"11",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"11",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"11",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"11",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"11",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"11",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -4319,19 +4445,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"12")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"12")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"12",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"12",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"12",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"12",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"12",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"12",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4351,19 +4477,19 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"13")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"13")</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"13",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"13",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"13",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"13",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"13",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"13",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -4383,19 +4509,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"14")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"14")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"14",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"14",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"14",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"14",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"14",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"14",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4415,19 +4541,19 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"15")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"15")</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"15",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"15",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"15",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"15",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"15",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"15",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -4447,19 +4573,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"16")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"16")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"16",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"16",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"16",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"16",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"16",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"16",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -4479,19 +4605,19 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"17")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"17")</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"17",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"17",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"17",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"17",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"17",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"17",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -4511,19 +4637,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"18")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"18")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"18",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"18",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"18",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"18",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"18",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"18",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -4543,19 +4669,19 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"19")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"19")</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"19",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"19",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"19",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"19",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"19",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"19",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -4575,19 +4701,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$77,"AX")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$80,"AX")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"AX",'Scénarios'!$I$2:$I$77,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"AX",'Scénarios'!$I$2:$I$80,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"AX",'Scénarios'!$I$2:$I$77,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"AX",'Scénarios'!$I$2:$I$80,"Réserve")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$77,"AX",'Scénarios'!$I$2:$I$77,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"AX",'Scénarios'!$I$2:$I$80,"KO")</f>
         <v/>
       </c>
       <c r="G21" s="10">

</xml_diff>

<commit_message>
Transport : application à part entière (NIMOVA · Transport)
Décision du gérant : le transport est un module comme Finance et AxisPro
Suite. Noyau : application « transport » (administration, direction,
finance, exploitation ; EGUITRA GROUP), liens des alertes et des constats
d'Analyse vers ses pages. Web : espace /transport (accent ambre) avec
tableau de bord, rotations, manquants, rentabilité, propriétaires et
répartition, taxes, flotte, routes et tarifs, paramètres ; écrans en
composants partagés ; registre, navigation, accueil, bascule, passerelle et
garde des pages ; /finance/transport redirige. Contrôle du tiers
propriétaire ou bénéficiaire (lisible, commun ou de la société), suite à
la revue de sécurité. Guides, dossier de conception, cahier de recette et
maquette d'API à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Cahier_de_recette.xlsx
+++ b/docs/projet/Cahier_de_recette.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scénarios'!$A$1:$L$81</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Scénarios'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3387,37 +3387,37 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>R62</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Exploitation</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Pilotage &gt; Trésorerie</t>
+          <t>Accueil NIMOVA &gt; Transport</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Afficher les flux mensuels et la prévision ; régler une échéance d'emprunt depuis une ligne de relevé.</t>
+          <t>Ouvrir l'application Transport depuis l'accueil, puis passer d'un menu à l'autre (Exploitation, Gestion, Référentiels) ; ouvrir l'ancienne adresse /finance/transport.</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>Emprunt repris</t>
+          <t>Compte exploitation et compte finance</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Encaissements, décaissements, cash net et solde par mois face au seuil ; échéance proposée au rapprochement, capital et intérêts comptabilisés une seule fois.</t>
+          <t>Application à part entière, aux couleurs du transport ; le parc ne voit pas Propriétaires et répartition ; l'ancienne adresse mène à l'application Transport.</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3429,37 +3429,37 @@
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>R62</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>AX</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Grille d'évaluation</t>
+          <t>Pilotage &gt; Trésorerie</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Importer l'outil de scoring du cabinet tel quel (version 3) ; le vérifier ; le mettre en vigueur.</t>
+          <t>Afficher les flux mensuels et la prévision ; régler une échéance d'emprunt depuis une ligne de relevé.</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Outil de scoring du cabinet (classeur)</t>
+          <t>Emprunt repris</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>7 gates et leurs règles (complétude minimale de 40 % au gate 1), 8 compartiments, 14 domaines, 104 critères (9 knock-outs), 39 pièces rattachées ; codes repris de la version précédente ; knock-out incomplet non bloquant, non applicable à 1 point ; version en vigueur.</t>
+          <t>Encaissements, décaissements, cash net et solde par mois face au seuil ; échéance proposée au rapprochement, capital et intérêts comptabilisés une seule fois.</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3471,7 +3471,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -3486,22 +3486,22 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>AxisPro &gt; Dossiers</t>
+          <t>AxisPro &gt; Grille d'évaluation</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Ouvrir un dossier.</t>
+          <t>Importer l'outil de scoring du cabinet tel quel (version 3) ; le vérifier ; le mettre en vigueur.</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>Projet réel anonymisé</t>
+          <t>Outil de scoring du cabinet (classeur)</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
+          <t>7 gates et leurs règles (complétude minimale de 40 % au gate 1), 8 compartiments, 14 domaines, 104 critères (9 knock-outs), 39 pièces rattachées ; codes repris de la version précédente ; knock-out incomplet non bloquant, non applicable à 1 point ; version en vigueur.</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3513,7 +3513,7 @@
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3528,22 +3528,22 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Évaluation</t>
+          <t>AxisPro &gt; Dossiers</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
+          <t>Ouvrir un dossier.</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Projet réel anonymisé</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
+          <t>Référence attribuée ; critères du premier gate à évaluer.</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3555,7 +3555,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Synthèse</t>
+          <t>Dossier &gt; Évaluation</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
+          <t>Évaluer les critères en saisie guidée ; déclarer disponible un knock-out sans pièce, puis lui joindre une preuve avec sa date de validité.</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
+          <t>Sans pièce, critère retenu « incomplet » (saisie inchangée) ; avec la preuve, retenu disponible ; Readiness, APD et Bankability recalculés ; pièce de la data room disponible.</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
@@ -3597,7 +3597,7 @@
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3612,12 +3612,12 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Comités</t>
+          <t>Dossier &gt; Synthèse</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
+          <t>Contrôler les knock-outs et les actions prioritaires ; passer au gate suivant ; forcer un passage refusé avec un motif.</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
+          <t>NO-GO si un knock-out est actif ; passage refusé avec ses motifs ; passage forcé inscrit au journal.</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3639,7 +3639,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -3654,12 +3654,12 @@
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Rapport</t>
+          <t>Dossier &gt; Comités</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
+          <t>Sceller et verrouiller une décision HOLD motivée ; vérifier l'empreinte ; tenter de modifier le dossier ; ouvrir une nouvelle révision ; comparer deux revues.</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
+          <t>Décision non modifiable, empreinte valide ; dossier figé jusqu'à la nouvelle révision ; comparaison des scores, gates et domaines.</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
@@ -3681,7 +3681,7 @@
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3696,22 +3696,22 @@
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Temps et facturation</t>
+          <t>Dossier &gt; Rapport</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Saisir des temps ; facturer les honoraires.</t>
+          <t>Télécharger le rapport du comité (PDF), le classeur d'évaluation, la fiche d'évaluation (la modifier puis la réimporter), la data room (.zip) et les pièces à fournir.</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>Taux horaire</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
+          <t>Politique appliquée et empreinte rappelées ; classeur au plan du modèle du cabinet ; import précédé d'un aperçu des changements.</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3723,7 +3723,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -3733,27 +3733,27 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Portail</t>
+          <t>Dossier &gt; Temps et facturation</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
+          <t>Saisir des temps ; facturer les honoraires.</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>Accès ouvert par le cabinet</t>
+          <t>Taux horaire</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
+          <t>Facture d'honoraires en brouillon dans la comptabilité du cabinet.</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -3765,7 +3765,7 @@
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3775,27 +3775,27 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Porteur de projet</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Data room</t>
+          <t>Portail</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
+          <t>Première connexion ; déposer une pièce ; écrire au cabinet.</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Accès ouvert par le cabinet</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
+          <t>Pièce visible du cabinet ; notes internes du cabinet invisibles du porteur.</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr"/>
@@ -3807,7 +3807,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>A09</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
@@ -3817,27 +3817,27 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Porteur de projet</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>Portail &gt; Pièces</t>
+          <t>Dossier &gt; Data room</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
+          <t>Valider une pièce ; en refuser une autre avec un motif.</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>Fichiers d'essai fournis par le prestataire</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
+          <t>Le porteur voit l'état de chaque pièce et le motif du refus.</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
@@ -3849,7 +3849,7 @@
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3859,27 +3859,27 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Direction (société du groupe seule)</t>
+          <t>Porteur de projet</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>AxisPro Suite</t>
+          <t>Portail &gt; Pièces</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
+          <t>Déposer un programme renommé en .pdf, puis un document Word à macros.</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fichiers d'essai fournis par le prestataire</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
+          <t>Dépôts refusés, formats acceptés rappelés (PDF, JPEG, PNG, DOCX, XLSX).</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3891,7 +3891,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A11</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -3901,27 +3901,27 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Direction (société du groupe seule)</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Synthèse, Évaluation</t>
+          <t>AxisPro Suite</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Confier deux compartiments à deux consultants ; filtrer la check-list sur « Mes compartiments » avec chacun.</t>
+          <t>Ouvrir AxisPro Suite avec un compte de direction ouvert à la seule société du groupe.</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>Deux comptes cabinet</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>Suivi par compartiment : score, critères, manques, études renseignées, consultant ; chaque consultant ne voit que ses critères ; changements inscrits au journal.</t>
+          <t>Aucun dossier, aucune pièce, revue ni grille du cabinet visible.</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr"/>
@@ -3933,7 +3933,7 @@
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3948,22 +3948,22 @@
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Dossier &gt; Stage gates</t>
+          <t>Dossier &gt; Synthèse, Évaluation</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>Évaluer quelques critères du gate 1 en dessous de 40 % de complétude, puis au-dessus.</t>
+          <t>Confier deux compartiments à deux consultants ; filtrer la check-list sur « Mes compartiments » avec chacun.</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Dossier ouvert</t>
+          <t>Deux comptes cabinet</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Gate 1 en HOLD avec le motif de complétude, puis GO ou CONDITIONAL GO selon le score.</t>
+          <t>Suivi par compartiment : score, critères, manques, études renseignées, consultant ; chaque consultant ne voit que ses critères ; changements inscrits au journal.</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>A14</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -3990,22 +3990,22 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Dossier &gt; Évaluation &gt; Importer une fiche</t>
+          <t>Dossier &gt; Stage gates</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Remplir l'outil de scoring du cabinet hors ligne (statuts, études à produire) et l'importer dans un dossier.</t>
+          <t>Évaluer quelques critères du gate 1 en dessous de 40 % de complétude, puis au-dessus.</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>Outil du cabinet rempli</t>
+          <t>Dossier ouvert</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>Aperçu des changements, puis statuts et études à produire repris ; notices de l'outil ignorées.</t>
+          <t>Gate 1 en HOLD avec le motif de complétude, puis GO ou CONDITIONAL GO selon le score.</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr"/>
@@ -4014,10 +4014,52 @@
       <c r="K80" s="6" t="inlineStr"/>
       <c r="L80" s="6" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>AX</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Dossier &gt; Évaluation &gt; Importer une fiche</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Remplir l'outil de scoring du cabinet hors ligne (statuts, études à produire) et l'importer dans un dossier.</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>Outil du cabinet rempli</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>Aperçu des changements, puis statuts et études à produire repris ; notices de l'outil ignorées.</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr"/>
+      <c r="I81" s="7" t="inlineStr"/>
+      <c r="J81" s="7" t="inlineStr"/>
+      <c r="K81" s="7" t="inlineStr"/>
+      <c r="L81" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L80"/>
+  <autoFilter ref="A1:L81"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
+    <dataValidation sqref="I2:I81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisir OK, KO ou Réserve." type="list">
       <formula1>"OK,KO,Réserve"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4093,19 +4135,19 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"1")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"1")</f>
         <v/>
       </c>
       <c r="D2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"1",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"1",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"1",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"1",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F2" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"1",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"1",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G2" s="9">
@@ -4125,19 +4167,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"2")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"2")</f>
         <v/>
       </c>
       <c r="D3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"2",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"2",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"2",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"2",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"2",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"2",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -4157,19 +4199,19 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"3")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"3")</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"3",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"3",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"3",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"3",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"3",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"3",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G4" s="9">
@@ -4189,19 +4231,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"4")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"4")</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"4",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"4",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"4",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"4",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"4",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"4",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -4221,19 +4263,19 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"5")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"5")</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"5",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"5",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"5",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"5",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"5",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"5",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G6" s="9">
@@ -4253,19 +4295,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"6")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"6")</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"6",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"6",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"6",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"6",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"6",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"6",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -4285,19 +4327,19 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"7")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"7")</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"7",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"7",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"7",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"7",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"7",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"7",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G8" s="9">
@@ -4317,19 +4359,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"8")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"8")</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"8",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"8",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"8",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"8",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"8",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"8",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -4349,19 +4391,19 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"9")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"9")</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"9",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"9",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"9",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"9",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"9",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"9",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G10" s="9">
@@ -4381,19 +4423,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"10")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"10")</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"10",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"10",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"10",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"10",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"10",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"10",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -4413,19 +4455,19 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"11")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"11")</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"11",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"11",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"11",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"11",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"11",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"11",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G12" s="9">
@@ -4445,19 +4487,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"12")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"12")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"12",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"12",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"12",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"12",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"12",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"12",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -4477,19 +4519,19 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"13")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"13")</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"13",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"13",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"13",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"13",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"13",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"13",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G14" s="9">
@@ -4509,19 +4551,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"14")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"14")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"14",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"14",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"14",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"14",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"14",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"14",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -4541,19 +4583,19 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"15")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"15")</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"15",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"15",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"15",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"15",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"15",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"15",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G16" s="9">
@@ -4573,19 +4615,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"16")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"16")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"16",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"16",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"16",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"16",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"16",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"16",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -4605,19 +4647,19 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"17")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"17")</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"17",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"17",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"17",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"17",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"17",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"17",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G18" s="9">
@@ -4637,19 +4679,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"18")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"18")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"18",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"18",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"18",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"18",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"18",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"18",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -4669,19 +4711,19 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"19")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"19")</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"19",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"19",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"19",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"19",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"19",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"19",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G20" s="9">
@@ -4701,19 +4743,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIF('Scénarios'!$B$2:$B$80,"AX")</f>
+        <f>COUNTIF('Scénarios'!$B$2:$B$81,"AX")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"AX",'Scénarios'!$I$2:$I$80,"OK")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"AX",'Scénarios'!$I$2:$I$81,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"AX",'Scénarios'!$I$2:$I$80,"Réserve")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"AX",'Scénarios'!$I$2:$I$81,"Réserve")</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>COUNTIFS('Scénarios'!$B$2:$B$80,"AX",'Scénarios'!$I$2:$I$80,"KO")</f>
+        <f>COUNTIFS('Scénarios'!$B$2:$B$81,"AX",'Scénarios'!$I$2:$I$81,"KO")</f>
         <v/>
       </c>
       <c r="G21" s="10">

</xml_diff>